<commit_message>
forgot to push the fixed dataset
</commit_message>
<xml_diff>
--- a/Datasets/Personal Workshop Data Records.xlsx
+++ b/Datasets/Personal Workshop Data Records.xlsx
@@ -94,51 +94,40 @@
     <t>[ARC9] BOCW Submachine Guns DLC</t>
   </si>
   <si>
-    <t xml:space="preserve">[ARC9] BOCW Tactical Rifles
-</t>
+    <t>[ARC9] BOCW Tactical Rifles</t>
   </si>
   <si>
-    <t xml:space="preserve">[ARC9] Multiplayer Camo Pack (Call of Duty: Black Ops Cold War)
-</t>
+    <t>[ARC9] Multiplayer Camo Pack (Call of Duty: Black Ops Cold War)</t>
   </si>
   <si>
-    <t xml:space="preserve">[ARC9] Zombies Camo Pack (Call of Duty: Black Ops Cold War)
-</t>
+    <t>[ARC9] Zombies Camo Pack (Call of Duty: Black Ops Cold War)</t>
   </si>
   <si>
-    <t xml:space="preserve">[BSMod] BOCW Finishing Moves
-</t>
+    <t>[BSMod] BOCW Finishing Moves</t>
   </si>
   <si>
     <t>Static</t>
   </si>
   <si>
-    <t xml:space="preserve">[ARC9] BOCW Light Machine Guns DLC (MG 82)
-</t>
+    <t>[ARC9] BOCW Light Machine Guns DLC (MG 82)</t>
   </si>
   <si>
-    <t xml:space="preserve">[ARC9] BOCW Melee (Knife)
-</t>
+    <t>[ARC9] BOCW Melee (Knife)</t>
   </si>
   <si>
-    <t xml:space="preserve">[ARC9] BOCW Special (M79)
-</t>
+    <t>[ARC9] BOCW Special (M79)</t>
   </si>
   <si>
-    <t xml:space="preserve">[ARC9] BOCW Tactical Rifles DLC (CARV.2)
-</t>
+    <t>[ARC9] BOCW Tactical Rifles DLC (CARV.2)</t>
   </si>
   <si>
-    <t xml:space="preserve">[ArcCW] .410 Ironhide (Call of Duty: Black Ops Cold War)
-</t>
+    <t>[ArcCW] .410 Ironhide (Call of Duty: Black Ops Cold War)</t>
   </si>
   <si>
-    <t xml:space="preserve">[ArcCW] AMP63 (Call of Duty: Black Ops Cold War)
-</t>
+    <t>[ArcCW] AMP63 (Call of Duty: Black Ops Cold War)</t>
   </si>
   <si>
-    <t xml:space="preserve">[ArcCW] AUG (Call of Duty: Black Ops Cold War)
-</t>
+    <t>[ArcCW] AUG (Call of Duty: Black Ops Cold War)</t>
   </si>
   <si>
     <t>[ArcCW] Ballistic Knife (Call of Duty: Black Ops Cold War)</t>
@@ -147,35 +136,28 @@
     <t>[ArcCW] C58 (Call of Duty: Black Ops Cold War)</t>
   </si>
   <si>
-    <t xml:space="preserve">[ArcCW] EM2 (Call of Duty: Black Ops Cold War)
-</t>
+    <t>[ArcCW] EM2 (Call of Duty: Black Ops Cold War)</t>
   </si>
   <si>
-    <t>[ArcCW] Gallo SA12 (Call of Duty: Black Ops Cold War</t>
+    <t>[ArcCW] Gallo SA12 (Call of Duty: Black Ops Cold War)</t>
   </si>
   <si>
-    <t xml:space="preserve">[ArcCW] KSP 45 (Call of Duty: Black Ops Cold War)
-</t>
+    <t>[ArcCW] KSP 45 (Call of Duty: Black Ops Cold War)</t>
   </si>
   <si>
-    <t xml:space="preserve">[ArcCW] LAPA (Call of Duty: Black Ops Cold War)
-</t>
+    <t>[ArcCW] LAPA (Call of Duty: Black Ops Cold War)</t>
   </si>
   <si>
-    <t xml:space="preserve">[ArcCW] Marshal (Call of Duty: Black Ops Cold War)
-</t>
+    <t>[ArcCW] Marshal (Call of Duty: Black Ops Cold War)</t>
   </si>
   <si>
-    <t xml:space="preserve">[ArcCW] MG 82 (Call of Duty: Black Ops Cold War)
-</t>
+    <t>[ArcCW] MG 82 (Call of Duty: Black Ops Cold War)</t>
   </si>
   <si>
-    <t xml:space="preserve">[ArcCW] OTs 9 (Call of Duty: Black Ops Cold War)
-</t>
+    <t>[ArcCW] OTs 9 (Call of Duty: Black Ops Cold War)</t>
   </si>
   <si>
-    <t xml:space="preserve">[ArcCW] ZRG 20mm (Call of Duty: Black Ops Cold War)
-</t>
+    <t>[ArcCW] ZRG 20mm (Call of Duty: Black Ops Cold War)</t>
   </si>
 </sst>
 </file>

</xml_diff>